<commit_message>
added AI slop checker (beta)
</commit_message>
<xml_diff>
--- a/docs/references/AI-Writing-Source-Register.xlsx
+++ b/docs/references/AI-Writing-Source-Register.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R3debdeae5feb4bc5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Extraction map" sheetId="2" r:id="Re1a6390966f74bf4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" r:id="R3aadfa0bd9824395"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Extraction map" sheetId="2" r:id="R2b07a34c9c4c42a4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17,7 +17,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
   </x:numFmts>
-  <x:fonts count="5">
+  <x:fonts count="6">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -42,6 +42,10 @@
     <x:font>
       <x:sz val="11"/>
       <x:color rgb="FF2251FF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
@@ -69,7 +73,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="14">
+  <x:cellXfs count="18">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -102,6 +106,16 @@
     <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -110,8 +124,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SourceRegister" displayName="SourceRegister" ref="A5:J26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:J26"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SourceRegister" displayName="SourceRegister" ref="A5:J29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:J29"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Family"/>
@@ -129,8 +143,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ExtractionMap" displayName="ExtractionMap" ref="A5:E258" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:E258"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ExtractionMap" displayName="ExtractionMap" ref="A5:E261" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:E261"/>
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Source item"/>
@@ -334,818 +348,914 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <sheetPr>
-    <tabColor rgb="FF051C2C"/>
-  </sheetPr>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="9" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="19" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="42" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="17" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="14" hidden="0" customWidth="1"/>
-    <col min="6" max="6" width="21" hidden="0" customWidth="1"/>
-    <col min="7" max="7" width="48" hidden="0" customWidth="1"/>
-    <col min="8" max="8" width="54" hidden="0" customWidth="1"/>
-    <col min="9" max="9" width="14" hidden="0" customWidth="1"/>
-    <col min="10" max="10" width="55" hidden="0" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="str">
-        <v>AI writing references | Rolling register</v>
-      </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
-    </row>
-    <row r="2">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-    </row>
-    <row r="3" ht="34" customHeight="1">
-      <c r="A3" s="4" t="str">
-        <v>21 sources • Reviewed 2 October 2026 • Filter by family or status. Add new rows inside the table; keep source IDs stable.</v>
-      </c>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
-      <c r="J4" s="1"/>
-    </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="7" t="str">
-        <v>ID</v>
-      </c>
-      <c r="B5" s="7" t="str">
-        <v>Family</v>
-      </c>
-      <c r="C5" s="7" t="str">
-        <v>Title</v>
-      </c>
-      <c r="D5" s="7" t="str">
-        <v>Type</v>
-      </c>
-      <c r="E5" s="7" t="str">
-        <v>Link</v>
-      </c>
-      <c r="F5" s="7" t="str">
-        <v>Review status</v>
-      </c>
-      <c r="G5" s="7" t="str">
-        <v>Extraction scope</v>
-      </c>
-      <c r="H5" s="7" t="str">
-        <v>Limits / next review</v>
-      </c>
-      <c r="I5" s="7" t="str">
-        <v>Reviewed</v>
-      </c>
-      <c r="J5" s="7" t="str">
-        <v>URL</v>
-      </c>
-    </row>
-    <row r="6" ht="100" customHeight="1">
-      <c r="A6" s="9" t="str">
-        <v>S01</v>
-      </c>
-      <c r="B6" s="9" t="str">
-        <v>Baseline</v>
-      </c>
-      <c r="C6" s="9" t="str">
-        <v>Wikipedia: Signs of AI writing</v>
-      </c>
-      <c r="D6" s="9" t="str">
-        <v>Supplied PDF</v>
-      </c>
-      <c r="E6" s="10" t="str">
-        <v>Open source</v>
-      </c>
-      <c r="F6" s="9" t="str">
-        <v>Included</v>
-      </c>
-      <c r="G6" s="9" t="str">
-        <v>47 supplied pages; original P001-P092 locators retained</v>
-      </c>
-      <c r="H6" s="9" t="str">
-        <v>Missing printed pages 48-51 are references, as confirmed by user. Local PDF controls the snapshot.</v>
-      </c>
-      <c r="I6" s="12" t="n">
-        <v>46297</v>
-      </c>
-      <c r="J6" s="9" t="str">
-        <v>https://en.wikipedia.org/wiki/Wikipedia:Signs_of_AI_writing</v>
-      </c>
-    </row>
-    <row r="7" ht="100" customHeight="1">
-      <c r="A7" s="8" t="str">
-        <v>S02</v>
-      </c>
-      <c r="B7" s="8" t="str">
-        <v>Baseline</v>
-      </c>
-      <c r="C7" s="8" t="str">
-        <v>Vale signs of AI writing</v>
-      </c>
-      <c r="D7" s="8" t="str">
-        <v>Repository</v>
-      </c>
-      <c r="E7" s="11" t="str">
-        <v>Open source</v>
-      </c>
-      <c r="F7" s="8" t="str">
-        <v>Included</v>
-      </c>
-      <c r="G7" s="8" t="str">
-        <v>18 rules and complete fixtures retained from original extraction</v>
-      </c>
-      <c r="H7" s="8" t="str">
-        <v>Pinned commit 305467bafd0e491c4c00e0196ef551e64eefc9c4; lint severity is not authorship confidence.</v>
-      </c>
-      <c r="I7" s="13" t="n">
-        <v>46297</v>
-      </c>
-      <c r="J7" s="8" t="str">
-        <v>https://github.com/ammil-industries/vale-signs-of-ai-writing</v>
-      </c>
-    </row>
-    <row r="8" ht="100" customHeight="1">
-      <c r="A8" s="9" t="str">
-        <v>S03</v>
-      </c>
-      <c r="B8" s="9" t="str">
-        <v>LAMP</v>
-      </c>
-      <c r="C8" s="9" t="str">
-        <v>Can AI writing be salvaged?</v>
-      </c>
-      <c r="D8" s="9" t="str">
-        <v>Paper</v>
-      </c>
-      <c r="E8" s="10" t="str">
-        <v>Open source</v>
-      </c>
-      <c r="F8" s="9" t="str">
-        <v>Included</v>
-      </c>
-      <c r="G8" s="9" t="str">
-        <v>Seven editorial categories and named subtypes</v>
-      </c>
-      <c r="H8" s="9" t="str">
-        <v>Creative-writing editing study; does not validate an authorship checklist.</v>
-      </c>
-      <c r="I8" s="12" t="n">
-        <v>46297</v>
-      </c>
-      <c r="J8" s="9" t="str">
-        <v>https://arxiv.org/html/2409.14509</v>
-      </c>
-    </row>
-    <row r="9" ht="100" customHeight="1">
-      <c r="A9" s="8" t="str">
-        <v>S04</v>
-      </c>
-      <c r="B9" s="8" t="str">
-        <v>LAMP</v>
-      </c>
-      <c r="C9" s="8" t="str">
-        <v>Writing Alignment / LAMP</v>
-      </c>
-      <c r="D9" s="8" t="str">
-        <v>Repository</v>
-      </c>
-      <c r="E9" s="11" t="str">
-        <v>Open source</v>
-      </c>
-      <c r="F9" s="8" t="str">
-        <v>Included</v>
-      </c>
-      <c r="G9" s="8" t="str">
-        <v>README, corpus schema and syntactic-data directory inspected</v>
-      </c>
-      <c r="H9" s="8" t="str">
-        <v>Corpus records and code not downloaded or executed; no claim to have classified every training example.</v>
-      </c>
-      <c r="I9" s="13" t="n">
-        <v>46297</v>
-      </c>
-      <c r="J9" s="8" t="str">
-        <v>https://github.com/salesforce/creativity_eval/tree/main/Writing_Alignment</v>
-      </c>
-    </row>
-    <row r="10" ht="100" customHeight="1">
-      <c r="A10" s="9" t="str">
-        <v>S05</v>
-      </c>
-      <c r="B10" s="9" t="str">
-        <v>Human Detectors</v>
-      </c>
-      <c r="C10" s="9" t="str">
-        <v>Human Detectors</v>
-      </c>
-      <c r="D10" s="9" t="str">
-        <v>Repository</v>
-      </c>
-      <c r="E10" s="10" t="str">
-        <v>Open source</v>
-      </c>
-      <c r="F10" s="9" t="str">
-        <v>Included</v>
-      </c>
-      <c r="G10" s="9" t="str">
-        <v>Detection guide and all 14 explanation categories</v>
-      </c>
-      <c r="H10" s="9" t="str">
-        <v>Expert observations include historical, contradictory and unsupported cues; preserved with qualifications.</v>
-      </c>
-      <c r="I10" s="12" t="n">
-        <v>46297</v>
-      </c>
-      <c r="J10" s="9" t="str">
-        <v>https://github.com/jenna-russell/human_detectors</v>
-      </c>
-    </row>
-    <row r="11" ht="100" customHeight="1">
-      <c r="A11" s="8" t="str">
-        <v>S06</v>
-      </c>
-      <c r="B11" s="8" t="str">
-        <v>Human Detectors</v>
-      </c>
-      <c r="C11" s="8" t="str">
-        <v>People who frequently use ChatGPT for writing tasks are accurate and robust detectors of AI-generated text</v>
-      </c>
-      <c r="D11" s="8" t="str">
-        <v>Paper</v>
-      </c>
-      <c r="E11" s="11" t="str">
-        <v>Open source</v>
-      </c>
-      <c r="F11" s="8" t="str">
-        <v>Context only</v>
-      </c>
-      <c r="G11" s="8" t="str">
-        <v>Research context for the repository guide</v>
-      </c>
-      <c r="H11" s="8" t="str">
-        <v>Individual heuristic validity does not follow from aggregate annotator performance.</v>
-      </c>
-      <c r="I11" s="13" t="n">
-        <v>46297</v>
-      </c>
-      <c r="J11" s="8" t="str">
-        <v>https://aclanthology.org/2025.acl-long.267/</v>
-      </c>
-    </row>
-    <row r="12" ht="100" customHeight="1">
-      <c r="A12" s="9" t="str">
-        <v>S07</v>
-      </c>
-      <c r="B12" s="9" t="str">
-        <v>Stop Slop</v>
-      </c>
-      <c r="C12" s="9" t="str">
-        <v>Stop Slop</v>
-      </c>
-      <c r="D12" s="9" t="str">
-        <v>Repository</v>
-      </c>
-      <c r="E12" s="10" t="str">
-        <v>Open source</v>
-      </c>
-      <c r="F12" s="9" t="str">
-        <v>Included</v>
-      </c>
-      <c r="G12" s="9" t="str">
-        <v>Writing instructions inspected online as source text; structures, phrases and five before/after examples</v>
-      </c>
-      <c r="H12" s="9" t="str">
-        <v>SKILL.md was not saved, installed or executed. Guidance rewritten; blanket stylistic bans are house preferences.</v>
-      </c>
-      <c r="I12" s="12" t="n">
-        <v>46297</v>
-      </c>
-      <c r="J12" s="9" t="str">
-        <v>https://github.com/hardikpandya/stop-slop</v>
-      </c>
-    </row>
-    <row r="13" ht="100" customHeight="1">
-      <c r="A13" s="8" t="str">
-        <v>S08</v>
-      </c>
-      <c r="B13" s="8" t="str">
-        <v>Measuring Slop</v>
-      </c>
-      <c r="C13" s="8" t="str">
-        <v>Measuring AI Slop in Text</v>
-      </c>
-      <c r="D13" s="8" t="str">
-        <v>Paper</v>
-      </c>
-      <c r="E13" s="11" t="str">
-        <v>Open source</v>
-      </c>
-      <c r="F13" s="8" t="str">
-        <v>Included</v>
-      </c>
-      <c r="G13" s="8" t="str">
-        <v>All 11 Appendix E codes; style and utility emphasis</v>
-      </c>
-      <c r="H13" s="8" t="str">
-        <v>Slop quality and machine authorship are different questions; factuality retained as context.</v>
-      </c>
-      <c r="I13" s="13" t="n">
-        <v>46297</v>
-      </c>
-      <c r="J13" s="8" t="str">
-        <v>https://arxiv.org/html/2509.19163v1</v>
-      </c>
-    </row>
-    <row r="14" ht="100" customHeight="1">
-      <c r="A14" s="9" t="str">
-        <v>S09</v>
-      </c>
-      <c r="B14" s="9" t="str">
-        <v>Cliche Highlighter</v>
-      </c>
-      <c r="C14" s="9" t="str">
-        <v>LLM cliché highlighter</v>
-      </c>
-      <c r="D14" s="9" t="str">
-        <v>Web tool</v>
-      </c>
-      <c r="E14" s="10" t="str">
-        <v>Open source</v>
-      </c>
-      <c r="F14" s="9" t="str">
-        <v>Included</v>
-      </c>
-      <c r="G14" s="9" t="str">
-        <v>All 39 named patterns in inspected implementation</v>
-      </c>
-      <c r="H14" s="9" t="str">
-        <v>Heuristic patterns, not a calibrated detector; includes ordinary rhetorical devices.</v>
-      </c>
-      <c r="I14" s="12" t="n">
-        <v>46297</v>
-      </c>
-      <c r="J14" s="9" t="str">
-        <v>https://tools.simonwillison.net/llm-cliche-highlighter</v>
-      </c>
-    </row>
-    <row r="15" ht="100" customHeight="1">
-      <c r="A15" s="8" t="str">
-        <v>S10</v>
-      </c>
-      <c r="B15" s="8" t="str">
-        <v>Cliche Highlighter</v>
-      </c>
-      <c r="C15" s="8" t="str">
-        <v>Highlighter source file</v>
-      </c>
-      <c r="D15" s="8" t="str">
-        <v>Repository file</v>
-      </c>
-      <c r="E15" s="11" t="str">
-        <v>Open source</v>
-      </c>
-      <c r="F15" s="8" t="str">
-        <v>Included</v>
-      </c>
-      <c r="G15" s="8" t="str">
-        <v>Read-only inspection of pattern definitions</v>
-      </c>
-      <c r="H15" s="8" t="str">
-        <v>No source code downloaded or executed; duplicates mapped to canonical entries.</v>
-      </c>
-      <c r="I15" s="13" t="n">
-        <v>46297</v>
-      </c>
-      <c r="J15" s="8" t="str">
-        <v>https://github.com/simonw/tools/blob/main/llm-cliche-highlighter.html</v>
-      </c>
-    </row>
-    <row r="16" ht="100" customHeight="1">
-      <c r="A16" s="9" t="str">
-        <v>S11</v>
-      </c>
-      <c r="B16" s="9" t="str">
-        <v>Prose Linter</v>
-      </c>
-      <c r="C16" s="9" t="str">
-        <v>slop prose linter</v>
-      </c>
-      <c r="D16" s="9" t="str">
-        <v>Repository</v>
-      </c>
-      <c r="E16" s="10" t="str">
-        <v>Open source</v>
-      </c>
-      <c r="F16" s="9" t="str">
-        <v>Included</v>
-      </c>
-      <c r="G16" s="9" t="str">
-        <v>All 118 rules in five indexed sets; full two vocabulary inventories</v>
-      </c>
-      <c r="H16" s="9" t="str">
-        <v>Small maintainer audits and domain-specific fits; default-branch snapshot can change.</v>
-      </c>
-      <c r="I16" s="12" t="n">
-        <v>46297</v>
-      </c>
-      <c r="J16" s="9" t="str">
-        <v>https://github.com/bheijden/slop</v>
-      </c>
-    </row>
-    <row r="17" ht="100" customHeight="1">
-      <c r="A17" s="8" t="str">
-        <v>S12</v>
-      </c>
-      <c r="B17" s="8" t="str">
-        <v>Reuters Institute</v>
-      </c>
-      <c r="C17" s="8" t="str">
-        <v>How AI-generated prose diverges from human writing and why it matters</v>
-      </c>
-      <c r="D17" s="8" t="str">
-        <v>Article</v>
-      </c>
-      <c r="E17" s="11" t="str">
-        <v>Open source</v>
-      </c>
-      <c r="F17" s="8" t="str">
-        <v>Included</v>
-      </c>
-      <c r="G17" s="8" t="str">
-        <v>Vocabulary, formulaic contrasts, generic claims and language convergence</v>
-      </c>
-      <c r="H17" s="8" t="str">
-        <v>Journalist interviews; human adoption of model-associated words weakens authorship inference.</v>
-      </c>
-      <c r="I17" s="13" t="n">
-        <v>46297</v>
-      </c>
-      <c r="J17" s="8" t="str">
-        <v>https://reutersinstitute.politics.ox.ac.uk/news/how-ai-generated-prose-diverges-human-writing-and-why-it-matters</v>
-      </c>
-    </row>
-    <row r="18" ht="100" customHeight="1">
-      <c r="A18" s="9" t="str">
-        <v>S13</v>
-      </c>
-      <c r="B18" s="9" t="str">
-        <v>Excess Vocabulary</v>
-      </c>
-      <c r="C18" s="9" t="str">
-        <v>Delving into LLM-assisted writing in biomedical publications through excess vocabulary</v>
-      </c>
-      <c r="D18" s="9" t="str">
-        <v>Paper</v>
-      </c>
-      <c r="E18" s="10" t="str">
-        <v>Open source</v>
-      </c>
-      <c r="F18" s="9" t="str">
-        <v>Included</v>
-      </c>
-      <c r="G18" s="9" t="str">
-        <v>Aggregate changes in style-word frequency and their limits</v>
-      </c>
-      <c r="H18" s="9" t="str">
-        <v>Biomedical abstracts, 2010-2024; population estimates are not individual-document verdicts.</v>
-      </c>
-      <c r="I18" s="12" t="n">
-        <v>46297</v>
-      </c>
-      <c r="J18" s="9" t="str">
-        <v>https://arxiv.org/html/2406.07016</v>
-      </c>
-    </row>
-    <row r="19" ht="100" customHeight="1">
-      <c r="A19" s="8" t="str">
-        <v>S14</v>
-      </c>
-      <c r="B19" s="8" t="str">
-        <v>HC3</v>
-      </c>
-      <c r="C19" s="8" t="str">
-        <v>How Close is ChatGPT to Human Experts?</v>
-      </c>
-      <c r="D19" s="8" t="str">
-        <v>Paper</v>
-      </c>
-      <c r="E19" s="11" t="str">
-        <v>Open source</v>
-      </c>
-      <c r="F19" s="8" t="str">
-        <v>Included</v>
-      </c>
-      <c r="G19" s="8" t="str">
-        <v>Sections 3.2 and 4: qualitative and linguistic differences</v>
-      </c>
-      <c r="H19" s="8" t="str">
-        <v>Early ChatGPT, English and Chinese Q&amp;A; direction can vary across languages and domains.</v>
-      </c>
-      <c r="I19" s="13" t="n">
-        <v>46297</v>
-      </c>
-      <c r="J19" s="8" t="str">
-        <v>https://arxiv.org/html/2301.07597</v>
-      </c>
-    </row>
-    <row r="20" ht="100" customHeight="1">
-      <c r="A20" s="9" t="str">
-        <v>S15</v>
-      </c>
-      <c r="B20" s="9" t="str">
-        <v>HC3</v>
-      </c>
-      <c r="C20" s="9" t="str">
-        <v>Human ChatGPT Comparison Corpus</v>
-      </c>
-      <c r="D20" s="9" t="str">
-        <v>Repository</v>
-      </c>
-      <c r="E20" s="10" t="str">
-        <v>Open source</v>
-      </c>
-      <c r="F20" s="9" t="str">
-        <v>Included</v>
-      </c>
-      <c r="G20" s="9" t="str">
-        <v>README and linguistic_analysis directory inspected</v>
-      </c>
-      <c r="H20" s="9" t="str">
-        <v>Training data not downloaded; linguistic_analysis directory is a placeholder, not a complete analysis package.</v>
-      </c>
-      <c r="I20" s="12" t="n">
-        <v>46297</v>
-      </c>
-      <c r="J20" s="9" t="str">
-        <v>https://github.com/Hello-SimpleAI/chatgpt-comparison-detection</v>
-      </c>
-    </row>
-    <row r="21" ht="100" customHeight="1">
-      <c r="A21" s="8" t="str">
-        <v>S16</v>
-      </c>
-      <c r="B21" s="8" t="str">
-        <v>MAGE</v>
-      </c>
-      <c r="C21" s="8" t="str">
-        <v>MAGE</v>
-      </c>
-      <c r="D21" s="8" t="str">
-        <v>Repository</v>
-      </c>
-      <c r="E21" s="11" t="str">
-        <v>Open source</v>
-      </c>
-      <c r="F21" s="8" t="str">
-        <v>Context only</v>
-      </c>
-      <c r="G21" s="8" t="str">
-        <v>Detector training and evaluation documentation</v>
-      </c>
-      <c r="H21" s="8" t="str">
-        <v>No explicit additional prose-tell taxonomy in inspected documentation; corpus labels are not editorial rules.</v>
-      </c>
-      <c r="I21" s="13" t="n">
-        <v>46297</v>
-      </c>
-      <c r="J21" s="8" t="str">
-        <v>https://github.com/yafuly/MAGE</v>
-      </c>
-    </row>
-    <row r="22" ht="100" customHeight="1">
-      <c r="A22" s="9" t="str">
-        <v>S17</v>
-      </c>
-      <c r="B22" s="9" t="str">
-        <v>MAGE</v>
-      </c>
-      <c r="C22" s="9" t="str">
-        <v>MAGE: Machine-generated Text Detection in the Wild</v>
-      </c>
-      <c r="D22" s="9" t="str">
-        <v>Paper</v>
-      </c>
-      <c r="E22" s="10" t="str">
-        <v>Open source</v>
-      </c>
-      <c r="F22" s="9" t="str">
-        <v>Context only</v>
-      </c>
-      <c r="G22" s="9" t="str">
-        <v>Benchmark scope and generalisation problem</v>
-      </c>
-      <c r="H22" s="9" t="str">
-        <v>Do not derive stylistic rules merely from a detector score or model architecture.</v>
-      </c>
-      <c r="I22" s="12" t="n">
-        <v>46297</v>
-      </c>
-      <c r="J22" s="9" t="str">
-        <v>https://aclanthology.org/2024.acl-long.3/</v>
-      </c>
-    </row>
-    <row r="23" ht="100" customHeight="1">
-      <c r="A23" s="8" t="str">
-        <v>S18</v>
-      </c>
-      <c r="B23" s="8" t="str">
-        <v>M4</v>
-      </c>
-      <c r="C23" s="8" t="str">
-        <v>M4</v>
-      </c>
-      <c r="D23" s="8" t="str">
-        <v>Repository</v>
-      </c>
-      <c r="E23" s="11" t="str">
-        <v>Open source</v>
-      </c>
-      <c r="F23" s="8" t="str">
-        <v>Context only</v>
-      </c>
-      <c r="G23" s="8" t="str">
-        <v>Multilingual and multi-domain detector resources</v>
-      </c>
-      <c r="H23" s="8" t="str">
-        <v>Classifier features do not establish a fixed direction or universal writing tell.</v>
-      </c>
-      <c r="I23" s="13" t="n">
-        <v>46297</v>
-      </c>
-      <c r="J23" s="8" t="str">
-        <v>https://github.com/mbzuai-nlp/M4</v>
-      </c>
-    </row>
-    <row r="24" ht="100" customHeight="1">
-      <c r="A24" s="9" t="str">
-        <v>S19</v>
-      </c>
-      <c r="B24" s="9" t="str">
-        <v>M4</v>
-      </c>
-      <c r="C24" s="9" t="str">
-        <v>M4: Multi-generator, Multi-domain, and Multi-lingual Black-Box Machine-Generated Text Detection</v>
-      </c>
-      <c r="D24" s="9" t="str">
-        <v>Paper</v>
-      </c>
-      <c r="E24" s="10" t="str">
-        <v>Open source</v>
-      </c>
-      <c r="F24" s="9" t="str">
-        <v>Context only</v>
-      </c>
-      <c r="G24" s="9" t="str">
-        <v>Benchmark scope and cross-domain limits</v>
-      </c>
-      <c r="H24" s="9" t="str">
-        <v>Retained for future research; no invented prose rules added.</v>
-      </c>
-      <c r="I24" s="12" t="n">
-        <v>46297</v>
-      </c>
-      <c r="J24" s="9" t="str">
-        <v>https://aclanthology.org/2024.eacl-long.83/</v>
-      </c>
-    </row>
-    <row r="25" ht="100" customHeight="1">
-      <c r="A25" s="8" t="str">
-        <v>S20</v>
-      </c>
-      <c r="B25" s="8" t="str">
-        <v>Measuring Slop</v>
-      </c>
-      <c r="C25" s="8" t="str">
-        <v>Measuring Slop companion repository</v>
-      </c>
-      <c r="D25" s="8" t="str">
-        <v>Repository</v>
-      </c>
-      <c r="E25" s="11" t="str">
-        <v>Open source</v>
-      </c>
-      <c r="F25" s="8" t="str">
-        <v>Unavailable corpus</v>
-      </c>
-      <c r="G25" s="8" t="str">
-        <v>Root inspected: README, license and gitignore</v>
-      </c>
-      <c r="H25" s="8" t="str">
-        <v>Linked repository currently provides no usable annotation corpus or rule catalog. Paper supplies the taxonomy.</v>
-      </c>
-      <c r="I25" s="13" t="n">
-        <v>46297</v>
-      </c>
-      <c r="J25" s="8" t="str">
-        <v>https://github.com/cshaib/slop</v>
-      </c>
-    </row>
-    <row r="26" ht="100" customHeight="1">
-      <c r="A26" s="9" t="str">
-        <v>S21</v>
-      </c>
-      <c r="B26" s="9" t="str">
-        <v>Excess Vocabulary</v>
-      </c>
-      <c r="C26" s="9" t="str">
-        <v>Excess vocabulary analysis and annotations</v>
-      </c>
-      <c r="D26" s="9" t="str">
-        <v>Repository</v>
-      </c>
-      <c r="E26" s="10" t="str">
-        <v>Open source</v>
-      </c>
-      <c r="F26" s="9" t="str">
-        <v>Included</v>
-      </c>
-      <c r="G26" s="9" t="str">
-        <v>All 407 style-labelled rows in results/excess_words.csv</v>
-      </c>
-      <c r="H26" s="9" t="str">
-        <v>Across all selected years, not the 2024-only list; compressed counts and analysis code not downloaded.</v>
-      </c>
-      <c r="I26" s="12" t="n">
-        <v>46297</v>
-      </c>
-      <c r="J26" s="9" t="str">
-        <v>https://github.com/berenslab/llm-excess-vocab</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells>
-    <mergeCell ref="A1:J2"/>
-    <mergeCell ref="A3:J3"/>
-  </mergeCells>
-  <dataValidations count="1">
-    <dataValidation type="list" sqref="F6:F1000">
-      <formula1>"Included,Context only,Unavailable corpus,Pending review"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <hyperlinks>
-    <hyperlink ref="E6" r:id="rIdSource1" display="Open source"/>
-    <hyperlink ref="E7" r:id="rIdSource2" display="Open source"/>
-    <hyperlink ref="E8" r:id="rIdSource3" display="Open source"/>
-    <hyperlink ref="E9" r:id="rIdSource4" display="Open source"/>
-    <hyperlink ref="E10" r:id="rIdSource5" display="Open source"/>
-    <hyperlink ref="E11" r:id="rIdSource6" display="Open source"/>
-    <hyperlink ref="E12" r:id="rIdSource7" display="Open source"/>
-    <hyperlink ref="E13" r:id="rIdSource8" display="Open source"/>
-    <hyperlink ref="E14" r:id="rIdSource9" display="Open source"/>
-    <hyperlink ref="E15" r:id="rIdSource10" display="Open source"/>
-    <hyperlink ref="E16" r:id="rIdSource11" display="Open source"/>
-    <hyperlink ref="E17" r:id="rIdSource12" display="Open source"/>
-    <hyperlink ref="E18" r:id="rIdSource13" display="Open source"/>
-    <hyperlink ref="E19" r:id="rIdSource14" display="Open source"/>
-    <hyperlink ref="E20" r:id="rIdSource15" display="Open source"/>
-    <hyperlink ref="E21" r:id="rIdSource16" display="Open source"/>
-    <hyperlink ref="E22" r:id="rIdSource17" display="Open source"/>
-    <hyperlink ref="E23" r:id="rIdSource18" display="Open source"/>
-    <hyperlink ref="E24" r:id="rIdSource19" display="Open source"/>
-    <hyperlink ref="E25" r:id="rIdSource20" display="Open source"/>
-    <hyperlink ref="E26" r:id="rIdSource21" display="Open source"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="R4aeb4afb26b1404e"/>
-  </tableParts>
-</worksheet>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FF051C2C"/>
+  </x:sheetPr>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="9" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="19" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="42" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="17" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="21" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="48" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="54" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="14" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="55" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="3" t="str">
+        <x:v>AI Slop Signatures source register</x:v>
+      </x:c>
+      <x:c r="B1" s="2"/>
+      <x:c r="C1" s="2"/>
+      <x:c r="D1" s="2"/>
+      <x:c r="E1" s="2"/>
+      <x:c r="F1" s="2"/>
+      <x:c r="G1" s="2"/>
+      <x:c r="H1" s="2"/>
+      <x:c r="I1" s="2"/>
+      <x:c r="J1" s="2"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="2"/>
+      <x:c r="B2" s="2"/>
+      <x:c r="C2" s="2"/>
+      <x:c r="D2" s="2"/>
+      <x:c r="E2" s="2"/>
+      <x:c r="F2" s="2"/>
+      <x:c r="G2" s="2"/>
+      <x:c r="H2" s="2"/>
+      <x:c r="I2" s="2"/>
+      <x:c r="J2" s="2"/>
+    </x:row>
+    <x:row r="3" ht="34" customHeight="1">
+      <x:c r="A3" s="4" t="str">
+        <x:v>24 sources. Updated 12 October 2026. Review dates apply to individual records. Keep source IDs stable.</x:v>
+      </x:c>
+      <x:c r="B3" s="1"/>
+      <x:c r="C3" s="1"/>
+      <x:c r="D3" s="1"/>
+      <x:c r="E3" s="1"/>
+      <x:c r="F3" s="1"/>
+      <x:c r="G3" s="1"/>
+      <x:c r="H3" s="1"/>
+      <x:c r="I3" s="1"/>
+      <x:c r="J3" s="1"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="1"/>
+      <x:c r="B4" s="1"/>
+      <x:c r="C4" s="1"/>
+      <x:c r="D4" s="1"/>
+      <x:c r="E4" s="1"/>
+      <x:c r="F4" s="1"/>
+      <x:c r="G4" s="1"/>
+      <x:c r="H4" s="1"/>
+      <x:c r="I4" s="1"/>
+      <x:c r="J4" s="1"/>
+    </x:row>
+    <x:row r="5" ht="30" customHeight="1">
+      <x:c r="A5" s="7" t="str">
+        <x:v>ID</x:v>
+      </x:c>
+      <x:c r="B5" s="7" t="str">
+        <x:v>Family</x:v>
+      </x:c>
+      <x:c r="C5" s="7" t="str">
+        <x:v>Title</x:v>
+      </x:c>
+      <x:c r="D5" s="7" t="str">
+        <x:v>Type</x:v>
+      </x:c>
+      <x:c r="E5" s="7" t="str">
+        <x:v>Link</x:v>
+      </x:c>
+      <x:c r="F5" s="7" t="str">
+        <x:v>Review status</x:v>
+      </x:c>
+      <x:c r="G5" s="7" t="str">
+        <x:v>Extraction scope</x:v>
+      </x:c>
+      <x:c r="H5" s="7" t="str">
+        <x:v>Limits / next review</x:v>
+      </x:c>
+      <x:c r="I5" s="7" t="str">
+        <x:v>Reviewed</x:v>
+      </x:c>
+      <x:c r="J5" s="7" t="str">
+        <x:v>URL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="100" customHeight="1">
+      <x:c r="A6" s="9" t="str">
+        <x:v>S01</x:v>
+      </x:c>
+      <x:c r="B6" s="9" t="str">
+        <x:v>Baseline</x:v>
+      </x:c>
+      <x:c r="C6" s="9" t="str">
+        <x:v>Wikipedia: Signs of AI writing</x:v>
+      </x:c>
+      <x:c r="D6" s="9" t="str">
+        <x:v>Supplied PDF</x:v>
+      </x:c>
+      <x:c r="E6" s="10" t="str">
+        <x:v>Open source</x:v>
+      </x:c>
+      <x:c r="F6" s="9" t="str">
+        <x:v>Included</x:v>
+      </x:c>
+      <x:c r="G6" s="9" t="str">
+        <x:v>47 supplied pages; original P001-P092 locators retained</x:v>
+      </x:c>
+      <x:c r="H6" s="9" t="str">
+        <x:v>Missing printed pages 48-51 are references, as confirmed by user. Local PDF controls the snapshot.</x:v>
+      </x:c>
+      <x:c r="I6" s="12" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="J6" s="9" t="str">
+        <x:v>https://en.wikipedia.org/wiki/Wikipedia:Signs_of_AI_writing</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="100" customHeight="1">
+      <x:c r="A7" s="8" t="str">
+        <x:v>S02</x:v>
+      </x:c>
+      <x:c r="B7" s="8" t="str">
+        <x:v>Baseline</x:v>
+      </x:c>
+      <x:c r="C7" s="8" t="str">
+        <x:v>Vale signs of AI writing</x:v>
+      </x:c>
+      <x:c r="D7" s="8" t="str">
+        <x:v>Repository</x:v>
+      </x:c>
+      <x:c r="E7" s="11" t="str">
+        <x:v>Open source</x:v>
+      </x:c>
+      <x:c r="F7" s="8" t="str">
+        <x:v>Included</x:v>
+      </x:c>
+      <x:c r="G7" s="8" t="str">
+        <x:v>18 rules and complete fixtures retained from original extraction</x:v>
+      </x:c>
+      <x:c r="H7" s="8" t="str">
+        <x:v>Pinned commit 305467bafd0e491c4c00e0196ef551e64eefc9c4; lint severity is not authorship confidence.</x:v>
+      </x:c>
+      <x:c r="I7" s="13" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="J7" s="8" t="str">
+        <x:v>https://github.com/ammil-industries/vale-signs-of-ai-writing</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="100" customHeight="1">
+      <x:c r="A8" s="9" t="str">
+        <x:v>S03</x:v>
+      </x:c>
+      <x:c r="B8" s="9" t="str">
+        <x:v>LAMP</x:v>
+      </x:c>
+      <x:c r="C8" s="9" t="str">
+        <x:v>Can AI writing be salvaged?</x:v>
+      </x:c>
+      <x:c r="D8" s="9" t="str">
+        <x:v>Paper</x:v>
+      </x:c>
+      <x:c r="E8" s="10" t="str">
+        <x:v>Open source</x:v>
+      </x:c>
+      <x:c r="F8" s="9" t="str">
+        <x:v>Included</x:v>
+      </x:c>
+      <x:c r="G8" s="9" t="str">
+        <x:v>Seven editorial categories and named subtypes</x:v>
+      </x:c>
+      <x:c r="H8" s="9" t="str">
+        <x:v>Creative-writing editing study; does not validate an authorship checklist.</x:v>
+      </x:c>
+      <x:c r="I8" s="12" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="J8" s="9" t="str">
+        <x:v>https://arxiv.org/html/2409.14509</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="100" customHeight="1">
+      <x:c r="A9" s="8" t="str">
+        <x:v>S04</x:v>
+      </x:c>
+      <x:c r="B9" s="8" t="str">
+        <x:v>LAMP</x:v>
+      </x:c>
+      <x:c r="C9" s="8" t="str">
+        <x:v>Writing Alignment / LAMP</x:v>
+      </x:c>
+      <x:c r="D9" s="8" t="str">
+        <x:v>Repository</x:v>
+      </x:c>
+      <x:c r="E9" s="11" t="str">
+        <x:v>Open source</x:v>
+      </x:c>
+      <x:c r="F9" s="8" t="str">
+        <x:v>Included</x:v>
+      </x:c>
+      <x:c r="G9" s="8" t="str">
+        <x:v>README, corpus schema and syntactic-data directory inspected</x:v>
+      </x:c>
+      <x:c r="H9" s="8" t="str">
+        <x:v>Corpus records and code not downloaded or executed; no claim to have classified every training example.</x:v>
+      </x:c>
+      <x:c r="I9" s="13" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="J9" s="8" t="str">
+        <x:v>https://github.com/salesforce/creativity_eval/tree/main/Writing_Alignment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="100" customHeight="1">
+      <x:c r="A10" s="9" t="str">
+        <x:v>S05</x:v>
+      </x:c>
+      <x:c r="B10" s="9" t="str">
+        <x:v>Human Detectors</x:v>
+      </x:c>
+      <x:c r="C10" s="9" t="str">
+        <x:v>Human Detectors</x:v>
+      </x:c>
+      <x:c r="D10" s="9" t="str">
+        <x:v>Repository</x:v>
+      </x:c>
+      <x:c r="E10" s="10" t="str">
+        <x:v>Open source</x:v>
+      </x:c>
+      <x:c r="F10" s="9" t="str">
+        <x:v>Included</x:v>
+      </x:c>
+      <x:c r="G10" s="9" t="str">
+        <x:v>Detection guide and all 14 explanation categories</x:v>
+      </x:c>
+      <x:c r="H10" s="9" t="str">
+        <x:v>Expert observations include historical, contradictory and unsupported cues; preserved with qualifications.</x:v>
+      </x:c>
+      <x:c r="I10" s="12" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="J10" s="9" t="str">
+        <x:v>https://github.com/jenna-russell/human_detectors</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="100" customHeight="1">
+      <x:c r="A11" s="8" t="str">
+        <x:v>S06</x:v>
+      </x:c>
+      <x:c r="B11" s="8" t="str">
+        <x:v>Human Detectors</x:v>
+      </x:c>
+      <x:c r="C11" s="8" t="str">
+        <x:v>People who frequently use ChatGPT for writing tasks are accurate and robust detectors of AI-generated text</x:v>
+      </x:c>
+      <x:c r="D11" s="8" t="str">
+        <x:v>Paper</x:v>
+      </x:c>
+      <x:c r="E11" s="11" t="str">
+        <x:v>Open source</x:v>
+      </x:c>
+      <x:c r="F11" s="8" t="str">
+        <x:v>Context only</x:v>
+      </x:c>
+      <x:c r="G11" s="8" t="str">
+        <x:v>Research context for the repository guide</x:v>
+      </x:c>
+      <x:c r="H11" s="8" t="str">
+        <x:v>Individual heuristic validity does not follow from aggregate annotator performance.</x:v>
+      </x:c>
+      <x:c r="I11" s="13" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="J11" s="8" t="str">
+        <x:v>https://aclanthology.org/2025.acl-long.267/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="100" customHeight="1">
+      <x:c r="A12" s="9" t="str">
+        <x:v>S07</x:v>
+      </x:c>
+      <x:c r="B12" s="9" t="str">
+        <x:v>Stop Slop</x:v>
+      </x:c>
+      <x:c r="C12" s="9" t="str">
+        <x:v>Stop Slop</x:v>
+      </x:c>
+      <x:c r="D12" s="9" t="str">
+        <x:v>Repository</x:v>
+      </x:c>
+      <x:c r="E12" s="10" t="str">
+        <x:v>Open source</x:v>
+      </x:c>
+      <x:c r="F12" s="9" t="str">
+        <x:v>Included</x:v>
+      </x:c>
+      <x:c r="G12" s="9" t="str">
+        <x:v>Writing instructions inspected online as source text; structures, phrases and five before/after examples</x:v>
+      </x:c>
+      <x:c r="H12" s="9" t="str">
+        <x:v>SKILL.md was not saved, installed or executed. Guidance rewritten; blanket stylistic bans are house preferences.</x:v>
+      </x:c>
+      <x:c r="I12" s="12" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="J12" s="9" t="str">
+        <x:v>https://github.com/hardikpandya/stop-slop</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="100" customHeight="1">
+      <x:c r="A13" s="8" t="str">
+        <x:v>S08</x:v>
+      </x:c>
+      <x:c r="B13" s="8" t="str">
+        <x:v>Measuring Slop</x:v>
+      </x:c>
+      <x:c r="C13" s="8" t="str">
+        <x:v>Measuring AI Slop in Text</x:v>
+      </x:c>
+      <x:c r="D13" s="8" t="str">
+        <x:v>Paper</x:v>
+      </x:c>
+      <x:c r="E13" s="11" t="str">
+        <x:v>Open source</x:v>
+      </x:c>
+      <x:c r="F13" s="8" t="str">
+        <x:v>Included</x:v>
+      </x:c>
+      <x:c r="G13" s="8" t="str">
+        <x:v>All 11 Appendix E codes; style and utility emphasis</x:v>
+      </x:c>
+      <x:c r="H13" s="8" t="str">
+        <x:v>Slop quality and machine authorship are different questions; factuality retained as context.</x:v>
+      </x:c>
+      <x:c r="I13" s="13" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="J13" s="8" t="str">
+        <x:v>https://arxiv.org/html/2509.19163v1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="100" customHeight="1">
+      <x:c r="A14" s="9" t="str">
+        <x:v>S09</x:v>
+      </x:c>
+      <x:c r="B14" s="9" t="str">
+        <x:v>Cliche Highlighter</x:v>
+      </x:c>
+      <x:c r="C14" s="9" t="str">
+        <x:v>LLM cliché highlighter</x:v>
+      </x:c>
+      <x:c r="D14" s="9" t="str">
+        <x:v>Web tool</x:v>
+      </x:c>
+      <x:c r="E14" s="10" t="str">
+        <x:v>Open source</x:v>
+      </x:c>
+      <x:c r="F14" s="9" t="str">
+        <x:v>Included</x:v>
+      </x:c>
+      <x:c r="G14" s="9" t="str">
+        <x:v>All 39 named patterns in inspected implementation</x:v>
+      </x:c>
+      <x:c r="H14" s="9" t="str">
+        <x:v>Heuristic patterns, not a calibrated detector; includes ordinary rhetorical devices.</x:v>
+      </x:c>
+      <x:c r="I14" s="12" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="J14" s="9" t="str">
+        <x:v>https://tools.simonwillison.net/llm-cliche-highlighter</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="100" customHeight="1">
+      <x:c r="A15" s="8" t="str">
+        <x:v>S10</x:v>
+      </x:c>
+      <x:c r="B15" s="8" t="str">
+        <x:v>Cliche Highlighter</x:v>
+      </x:c>
+      <x:c r="C15" s="8" t="str">
+        <x:v>Highlighter source file</x:v>
+      </x:c>
+      <x:c r="D15" s="8" t="str">
+        <x:v>Repository file</x:v>
+      </x:c>
+      <x:c r="E15" s="11" t="str">
+        <x:v>Open source</x:v>
+      </x:c>
+      <x:c r="F15" s="8" t="str">
+        <x:v>Included</x:v>
+      </x:c>
+      <x:c r="G15" s="8" t="str">
+        <x:v>Read-only inspection of pattern definitions</x:v>
+      </x:c>
+      <x:c r="H15" s="8" t="str">
+        <x:v>No source code downloaded or executed; duplicates mapped to canonical entries.</x:v>
+      </x:c>
+      <x:c r="I15" s="13" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="J15" s="8" t="str">
+        <x:v>https://github.com/simonw/tools/blob/main/llm-cliche-highlighter.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="100" customHeight="1">
+      <x:c r="A16" s="9" t="str">
+        <x:v>S11</x:v>
+      </x:c>
+      <x:c r="B16" s="9" t="str">
+        <x:v>Prose Linter</x:v>
+      </x:c>
+      <x:c r="C16" s="9" t="str">
+        <x:v>slop prose linter</x:v>
+      </x:c>
+      <x:c r="D16" s="9" t="str">
+        <x:v>Repository</x:v>
+      </x:c>
+      <x:c r="E16" s="10" t="str">
+        <x:v>Open source</x:v>
+      </x:c>
+      <x:c r="F16" s="9" t="str">
+        <x:v>Included</x:v>
+      </x:c>
+      <x:c r="G16" s="9" t="str">
+        <x:v>All 118 rules in five indexed sets; full two vocabulary inventories</x:v>
+      </x:c>
+      <x:c r="H16" s="9" t="str">
+        <x:v>Small maintainer audits and domain-specific fits; default-branch snapshot can change.</x:v>
+      </x:c>
+      <x:c r="I16" s="12" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="J16" s="9" t="str">
+        <x:v>https://github.com/bheijden/slop</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="100" customHeight="1">
+      <x:c r="A17" s="8" t="str">
+        <x:v>S12</x:v>
+      </x:c>
+      <x:c r="B17" s="8" t="str">
+        <x:v>Reuters Institute</x:v>
+      </x:c>
+      <x:c r="C17" s="8" t="str">
+        <x:v>How AI-generated prose diverges from human writing and why it matters</x:v>
+      </x:c>
+      <x:c r="D17" s="8" t="str">
+        <x:v>Article</x:v>
+      </x:c>
+      <x:c r="E17" s="11" t="str">
+        <x:v>Open source</x:v>
+      </x:c>
+      <x:c r="F17" s="8" t="str">
+        <x:v>Included</x:v>
+      </x:c>
+      <x:c r="G17" s="8" t="str">
+        <x:v>Vocabulary, formulaic contrasts, generic claims and language convergence</x:v>
+      </x:c>
+      <x:c r="H17" s="8" t="str">
+        <x:v>Journalist interviews; human adoption of model-associated words weakens authorship inference.</x:v>
+      </x:c>
+      <x:c r="I17" s="13" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="J17" s="8" t="str">
+        <x:v>https://reutersinstitute.politics.ox.ac.uk/news/how-ai-generated-prose-diverges-human-writing-and-why-it-matters</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="100" customHeight="1">
+      <x:c r="A18" s="9" t="str">
+        <x:v>S13</x:v>
+      </x:c>
+      <x:c r="B18" s="9" t="str">
+        <x:v>Excess Vocabulary</x:v>
+      </x:c>
+      <x:c r="C18" s="9" t="str">
+        <x:v>Delving into LLM-assisted writing in biomedical publications through excess vocabulary</x:v>
+      </x:c>
+      <x:c r="D18" s="9" t="str">
+        <x:v>Paper</x:v>
+      </x:c>
+      <x:c r="E18" s="10" t="str">
+        <x:v>Open source</x:v>
+      </x:c>
+      <x:c r="F18" s="9" t="str">
+        <x:v>Included</x:v>
+      </x:c>
+      <x:c r="G18" s="9" t="str">
+        <x:v>Aggregate changes in style-word frequency and their limits</x:v>
+      </x:c>
+      <x:c r="H18" s="9" t="str">
+        <x:v>Biomedical abstracts, 2010-2024; population estimates are not individual-document verdicts.</x:v>
+      </x:c>
+      <x:c r="I18" s="12" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="J18" s="9" t="str">
+        <x:v>https://arxiv.org/html/2406.07016</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="100" customHeight="1">
+      <x:c r="A19" s="8" t="str">
+        <x:v>S14</x:v>
+      </x:c>
+      <x:c r="B19" s="8" t="str">
+        <x:v>HC3</x:v>
+      </x:c>
+      <x:c r="C19" s="8" t="str">
+        <x:v>How Close is ChatGPT to Human Experts?</x:v>
+      </x:c>
+      <x:c r="D19" s="8" t="str">
+        <x:v>Paper</x:v>
+      </x:c>
+      <x:c r="E19" s="11" t="str">
+        <x:v>Open source</x:v>
+      </x:c>
+      <x:c r="F19" s="8" t="str">
+        <x:v>Included</x:v>
+      </x:c>
+      <x:c r="G19" s="8" t="str">
+        <x:v>Sections 3.2 and 4: qualitative and linguistic differences</x:v>
+      </x:c>
+      <x:c r="H19" s="8" t="str">
+        <x:v>Early ChatGPT, English and Chinese Q&amp;A; direction can vary across languages and domains.</x:v>
+      </x:c>
+      <x:c r="I19" s="13" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="J19" s="8" t="str">
+        <x:v>https://arxiv.org/html/2301.07597</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="100" customHeight="1">
+      <x:c r="A20" s="9" t="str">
+        <x:v>S15</x:v>
+      </x:c>
+      <x:c r="B20" s="9" t="str">
+        <x:v>HC3</x:v>
+      </x:c>
+      <x:c r="C20" s="9" t="str">
+        <x:v>Human ChatGPT Comparison Corpus</x:v>
+      </x:c>
+      <x:c r="D20" s="9" t="str">
+        <x:v>Repository</x:v>
+      </x:c>
+      <x:c r="E20" s="10" t="str">
+        <x:v>Open source</x:v>
+      </x:c>
+      <x:c r="F20" s="9" t="str">
+        <x:v>Included</x:v>
+      </x:c>
+      <x:c r="G20" s="9" t="str">
+        <x:v>README and linguistic_analysis directory inspected</x:v>
+      </x:c>
+      <x:c r="H20" s="9" t="str">
+        <x:v>Training data not downloaded; linguistic_analysis directory is a placeholder, not a complete analysis package.</x:v>
+      </x:c>
+      <x:c r="I20" s="12" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="J20" s="9" t="str">
+        <x:v>https://github.com/Hello-SimpleAI/chatgpt-comparison-detection</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="100" customHeight="1">
+      <x:c r="A21" s="8" t="str">
+        <x:v>S16</x:v>
+      </x:c>
+      <x:c r="B21" s="8" t="str">
+        <x:v>MAGE</x:v>
+      </x:c>
+      <x:c r="C21" s="8" t="str">
+        <x:v>MAGE</x:v>
+      </x:c>
+      <x:c r="D21" s="8" t="str">
+        <x:v>Repository</x:v>
+      </x:c>
+      <x:c r="E21" s="11" t="str">
+        <x:v>Open source</x:v>
+      </x:c>
+      <x:c r="F21" s="8" t="str">
+        <x:v>Context only</x:v>
+      </x:c>
+      <x:c r="G21" s="8" t="str">
+        <x:v>Detector training and evaluation documentation</x:v>
+      </x:c>
+      <x:c r="H21" s="8" t="str">
+        <x:v>No explicit additional prose-tell taxonomy in inspected documentation; corpus labels are not editorial rules.</x:v>
+      </x:c>
+      <x:c r="I21" s="13" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="J21" s="8" t="str">
+        <x:v>https://github.com/yafuly/MAGE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="100" customHeight="1">
+      <x:c r="A22" s="9" t="str">
+        <x:v>S17</x:v>
+      </x:c>
+      <x:c r="B22" s="9" t="str">
+        <x:v>MAGE</x:v>
+      </x:c>
+      <x:c r="C22" s="9" t="str">
+        <x:v>MAGE: Machine-generated Text Detection in the Wild</x:v>
+      </x:c>
+      <x:c r="D22" s="9" t="str">
+        <x:v>Paper</x:v>
+      </x:c>
+      <x:c r="E22" s="10" t="str">
+        <x:v>Open source</x:v>
+      </x:c>
+      <x:c r="F22" s="9" t="str">
+        <x:v>Context only</x:v>
+      </x:c>
+      <x:c r="G22" s="9" t="str">
+        <x:v>Benchmark scope and generalisation problem</x:v>
+      </x:c>
+      <x:c r="H22" s="9" t="str">
+        <x:v>Do not derive stylistic rules merely from a detector score or model architecture.</x:v>
+      </x:c>
+      <x:c r="I22" s="12" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="J22" s="9" t="str">
+        <x:v>https://aclanthology.org/2024.acl-long.3/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="100" customHeight="1">
+      <x:c r="A23" s="8" t="str">
+        <x:v>S18</x:v>
+      </x:c>
+      <x:c r="B23" s="8" t="str">
+        <x:v>M4</x:v>
+      </x:c>
+      <x:c r="C23" s="8" t="str">
+        <x:v>M4</x:v>
+      </x:c>
+      <x:c r="D23" s="8" t="str">
+        <x:v>Repository</x:v>
+      </x:c>
+      <x:c r="E23" s="11" t="str">
+        <x:v>Open source</x:v>
+      </x:c>
+      <x:c r="F23" s="8" t="str">
+        <x:v>Context only</x:v>
+      </x:c>
+      <x:c r="G23" s="8" t="str">
+        <x:v>Multilingual and multi-domain detector resources</x:v>
+      </x:c>
+      <x:c r="H23" s="8" t="str">
+        <x:v>Classifier features do not establish a fixed direction or universal writing tell.</x:v>
+      </x:c>
+      <x:c r="I23" s="13" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="J23" s="8" t="str">
+        <x:v>https://github.com/mbzuai-nlp/M4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="100" customHeight="1">
+      <x:c r="A24" s="9" t="str">
+        <x:v>S19</x:v>
+      </x:c>
+      <x:c r="B24" s="9" t="str">
+        <x:v>M4</x:v>
+      </x:c>
+      <x:c r="C24" s="9" t="str">
+        <x:v>M4: Multi-generator, Multi-domain, and Multi-lingual Black-Box Machine-Generated Text Detection</x:v>
+      </x:c>
+      <x:c r="D24" s="9" t="str">
+        <x:v>Paper</x:v>
+      </x:c>
+      <x:c r="E24" s="10" t="str">
+        <x:v>Open source</x:v>
+      </x:c>
+      <x:c r="F24" s="9" t="str">
+        <x:v>Context only</x:v>
+      </x:c>
+      <x:c r="G24" s="9" t="str">
+        <x:v>Benchmark scope and cross-domain limits</x:v>
+      </x:c>
+      <x:c r="H24" s="9" t="str">
+        <x:v>Retained for future research; no invented prose rules added.</x:v>
+      </x:c>
+      <x:c r="I24" s="12" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="J24" s="9" t="str">
+        <x:v>https://aclanthology.org/2024.eacl-long.83/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="100" customHeight="1">
+      <x:c r="A25" s="8" t="str">
+        <x:v>S20</x:v>
+      </x:c>
+      <x:c r="B25" s="8" t="str">
+        <x:v>Measuring Slop</x:v>
+      </x:c>
+      <x:c r="C25" s="8" t="str">
+        <x:v>Measuring Slop companion repository</x:v>
+      </x:c>
+      <x:c r="D25" s="8" t="str">
+        <x:v>Repository</x:v>
+      </x:c>
+      <x:c r="E25" s="11" t="str">
+        <x:v>Open source</x:v>
+      </x:c>
+      <x:c r="F25" s="8" t="str">
+        <x:v>Unavailable corpus</x:v>
+      </x:c>
+      <x:c r="G25" s="8" t="str">
+        <x:v>Root inspected: README, license and gitignore</x:v>
+      </x:c>
+      <x:c r="H25" s="8" t="str">
+        <x:v>Linked repository currently provides no usable annotation corpus or rule catalog. Paper supplies the taxonomy.</x:v>
+      </x:c>
+      <x:c r="I25" s="13" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="J25" s="8" t="str">
+        <x:v>https://github.com/cshaib/slop</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="100" customHeight="1">
+      <x:c r="A26" s="9" t="str">
+        <x:v>S21</x:v>
+      </x:c>
+      <x:c r="B26" s="9" t="str">
+        <x:v>Excess Vocabulary</x:v>
+      </x:c>
+      <x:c r="C26" s="9" t="str">
+        <x:v>Excess vocabulary analysis and annotations</x:v>
+      </x:c>
+      <x:c r="D26" s="9" t="str">
+        <x:v>Repository</x:v>
+      </x:c>
+      <x:c r="E26" s="10" t="str">
+        <x:v>Open source</x:v>
+      </x:c>
+      <x:c r="F26" s="9" t="str">
+        <x:v>Included</x:v>
+      </x:c>
+      <x:c r="G26" s="9" t="str">
+        <x:v>All 407 style-labelled rows in results/excess_words.csv</x:v>
+      </x:c>
+      <x:c r="H26" s="9" t="str">
+        <x:v>Across all selected years, not the 2024-only list; compressed counts and analysis code not downloaded.</x:v>
+      </x:c>
+      <x:c r="I26" s="12" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="J26" s="9" t="str">
+        <x:v>https://github.com/berenslab/llm-excess-vocab</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="84" customHeight="1">
+      <x:c r="A27" s="16" t="str">
+        <x:v>S22</x:v>
+      </x:c>
+      <x:c r="B27" s="16" t="str">
+        <x:v>Graphite</x:v>
+      </x:c>
+      <x:c r="C27" s="16" t="str">
+        <x:v>Graphite: AI Tells</x:v>
+      </x:c>
+      <x:c r="D27" s="16" t="str">
+        <x:v>Article</x:v>
+      </x:c>
+      <x:c r="E27" s="16" t="str">
+        <x:v>See URL at right</x:v>
+      </x:c>
+      <x:c r="F27" s="16" t="str">
+        <x:v>Included</x:v>
+      </x:c>
+      <x:c r="G27" s="16" t="str">
+        <x:v>Phrase variants and selected model-versus-human measurements; see the master concordance.</x:v>
+      </x:c>
+      <x:c r="H27" s="16" t="str">
+        <x:v>Rates describe matched web-article samples, not authorship probabilities.</x:v>
+      </x:c>
+      <x:c r="I27" s="17" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="J27" s="16" t="str">
+        <x:v>https://graphite.io/five-percent/research/ai-tells</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="84" customHeight="1">
+      <x:c r="A28" s="16" t="str">
+        <x:v>S23</x:v>
+      </x:c>
+      <x:c r="B28" s="16" t="str">
+        <x:v>Graphite</x:v>
+      </x:c>
+      <x:c r="C28" s="16" t="str">
+        <x:v>Graphite: AI Tells: Opus 5.5 Update</x:v>
+      </x:c>
+      <x:c r="D28" s="16" t="str">
+        <x:v>Article</x:v>
+      </x:c>
+      <x:c r="E28" s="16" t="str">
+        <x:v>See URL at right</x:v>
+      </x:c>
+      <x:c r="F28" s="16" t="str">
+        <x:v>Included</x:v>
+      </x:c>
+      <x:c r="G28" s="16" t="str">
+        <x:v>Additional phrase variants and selected comparisons between models.</x:v>
+      </x:c>
+      <x:c r="H28" s="16" t="str">
+        <x:v>A model-to-model ratio is not a human-relative rate.</x:v>
+      </x:c>
+      <x:c r="I28" s="17" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="J28" s="16" t="str">
+        <x:v>https://graphite.io/five-percent/research/ai-tells-opus-5-5-update</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="84" customHeight="1">
+      <x:c r="A29" s="16" t="str">
+        <x:v>S24</x:v>
+      </x:c>
+      <x:c r="B29" s="16" t="str">
+        <x:v>Punctuation</x:v>
+      </x:c>
+      <x:c r="C29" s="16" t="str">
+        <x:v>Devapratim Mohanty: The Story of the Omnipresent Hyphen</x:v>
+      </x:c>
+      <x:c r="D29" s="16" t="str">
+        <x:v>Commentary</x:v>
+      </x:c>
+      <x:c r="E29" s="16" t="str">
+        <x:v>See URL at right</x:v>
+      </x:c>
+      <x:c r="F29" s="16" t="str">
+        <x:v>Included</x:v>
+      </x:c>
+      <x:c r="G29" s="16" t="str">
+        <x:v>P144: unnecessary hyphens, with original examples based on user-supplied cases.</x:v>
+      </x:c>
+      <x:c r="H29" s="16" t="str">
+        <x:v>No measured frequency. Screenshot examples are not in the inspected article; proposed tokenization cause not treated as established.</x:v>
+      </x:c>
+      <x:c r="I29" s="17" t="d">
+        <x:v>2026-10-12T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="J29" s="16" t="str">
+        <x:v>https://medium.com/@devapratimm/the-story-of-the-omnipresent-hyphen-why-ai-cant-get-punctuation-right-b26e88426bad</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:J2"/>
+    <x:mergeCell ref="A3:J3"/>
+  </x:mergeCells>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="F6:F1000">
+      <x:formula1>"Included,Context only,Unavailable corpus,Pending review"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:hyperlinks>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="R333ab91df95b4742"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="R4edb8ef714de4dc4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="Rcfde7ccc84b9407c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="Re761dcac2e044e4e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="Ra3843117786b41db"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="R805d2de34ada43ec"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="R98f8a67e486b4ba5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="R86b6be964d6e4691"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="Rb73b45cec9c44c51"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="Ra801c792ef5a469b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="Rd404f5cc161b40e7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="R8c76127b5a824214"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="Rb33cfc3102de46b6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="R64201cacb80242a1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="R3857512a94864d6d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="Ra3f032f896dd4339"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="R71623b4c78b84422"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="R34d08a680b4a4093"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="Rec1fce3b3fcd4ce3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="Rd829d87600bf4ae7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="R0e8149b3eff34d52"/>
+  </x:hyperlinks>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb4e8d967d3b14da6"/>
+  </x:tableParts>
+</x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1180,7 +1290,7 @@
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>253 source items • P001–P138 refer to the master document. Repeated IDs are deliberate merges. Numeric thresholds are unvalidated source settings.</x:v>
+        <x:v>256 source-item records. Stable catalogue IDs link to the master reference; repeated IDs are deliberate.</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -5510,6 +5620,57 @@
       </x:c>
       <x:c r="E258" s="9" t="str">
         <x:v>Not a numeric rule</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="259" ht="60" customHeight="1">
+      <x:c r="A259" s="16" t="str">
+        <x:v>S22</x:v>
+      </x:c>
+      <x:c r="B259" s="16" t="str">
+        <x:v>Phrase observations and web-article comparisons</x:v>
+      </x:c>
+      <x:c r="C259" s="16" t="str">
+        <x:v>P139-P143 and merged examples</x:v>
+      </x:c>
+      <x:c r="D259" s="16" t="str">
+        <x:v>Grouped with existing entries; see master reconciliation</x:v>
+      </x:c>
+      <x:c r="E259" s="16" t="str">
+        <x:v>Only exact supported comparisons displayed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="260" ht="60" customHeight="1">
+      <x:c r="A260" s="16" t="str">
+        <x:v>S23</x:v>
+      </x:c>
+      <x:c r="B260" s="16" t="str">
+        <x:v>Updated phrase observations and model comparisons</x:v>
+      </x:c>
+      <x:c r="C260" s="16" t="str">
+        <x:v>P139-P143 and merged examples</x:v>
+      </x:c>
+      <x:c r="D260" s="16" t="str">
+        <x:v>Merged with S22; preserve model comparator</x:v>
+      </x:c>
+      <x:c r="E260" s="16" t="str">
+        <x:v>Model-to-model measurements are not human-relative</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="261" ht="60" customHeight="1">
+      <x:c r="A261" s="16" t="str">
+        <x:v>S24</x:v>
+      </x:c>
+      <x:c r="B261" s="16" t="str">
+        <x:v>Unnecessary hyphens</x:v>
+      </x:c>
+      <x:c r="C261" s="16" t="str">
+        <x:v>P144</x:v>
+      </x:c>
+      <x:c r="D261" s="16" t="str">
+        <x:v>Original examples; commentary listed as source</x:v>
+      </x:c>
+      <x:c r="E261" s="16" t="str">
+        <x:v>Spelling context matters; no prevalence estimate</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5519,7 +5680,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb6a2d1057bee4550"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11f5c5d859bf4777"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>